<commit_message>
Upload automático via Dashboard: 03 - Mar 2026.xlsx
</commit_message>
<xml_diff>
--- a/historico_dados/03 - Mar 2026.xlsx
+++ b/historico_dados/03 - Mar 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JFMELO\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F335650-1C94-4361-A851-9C1FD22E5A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DD2604-5AD0-42C3-A5BF-5BAA5DF7C36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="729" firstSheet="1" activeTab="5" xr2:uid="{BDCD7524-1CC9-4D12-94EE-1D81A0CE0740}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="729" firstSheet="2" activeTab="7" xr2:uid="{BDCD7524-1CC9-4D12-94EE-1D81A0CE0740}"/>
   </bookViews>
   <sheets>
     <sheet name="TURNOS" sheetId="16" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="243">
   <si>
     <t>DESCRIÇÃO</t>
   </si>
@@ -1139,12 +1139,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1232,15 +1232,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="23" formatCode="h:mm\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1582,6 +1573,15 @@
       </fill>
       <protection locked="0" hidden="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1606,14 +1606,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9CB1CAD2-0991-4AFA-A8C5-85F5500ACC1A}" name="tblTurnos" displayName="tblTurnos" ref="A2:E5" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63" tableBorderDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9CB1CAD2-0991-4AFA-A8C5-85F5500ACC1A}" name="tblTurnos" displayName="tblTurnos" ref="A2:E5" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60" tableBorderDxfId="59">
   <autoFilter ref="A2:E5" xr:uid="{9CB1CAD2-0991-4AFA-A8C5-85F5500ACC1A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{66C8A751-944C-4ED0-9B93-7EF7890BAC2C}" name="ID_TURNO" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{CE79B6B8-84BE-42CD-8597-D513FB5454F3}" name="TURNO" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{72B36434-A91F-4B46-ABFB-CA8660948243}" name="HORARIO_INICIO" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{39895036-CC40-4170-867E-4FB900291AD1}" name="HORARIO_FIM" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{883890C6-E58B-43F9-93BF-FE0182EAC856}" name="DESCRICAO" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{66C8A751-944C-4ED0-9B93-7EF7890BAC2C}" name="ID_TURNO" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{CE79B6B8-84BE-42CD-8597-D513FB5454F3}" name="TURNO" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{72B36434-A91F-4B46-ABFB-CA8660948243}" name="HORARIO_INICIO" dataDxfId="56"/>
+    <tableColumn id="4" xr3:uid="{39895036-CC40-4170-867E-4FB900291AD1}" name="HORARIO_FIM" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{883890C6-E58B-43F9-93BF-FE0182EAC856}" name="DESCRICAO" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1669,35 +1669,35 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{43641B7E-1E4B-4F99-8245-A48C23AE54BB}" name="tblModalidades" displayName="tblModalidades" ref="A2:D4" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{43641B7E-1E4B-4F99-8245-A48C23AE54BB}" name="tblModalidades" displayName="tblModalidades" ref="A2:D4" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="A2:D4" xr:uid="{43641B7E-1E4B-4F99-8245-A48C23AE54BB}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{B42A8C1C-387F-4E3D-A54F-CF1D913A6676}" name="ID_MODALIDADE" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{409E0C8E-C00D-45B9-8113-E86B37049A97}" name="MODALIDADE" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{9B83D5E8-C0D6-41D3-A5EB-27263A3A1DDA}" name="TIPO" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{D7FE0EEE-44EA-4C6B-B889-B4C030F1B758}" name=" DESCRICAO" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{B42A8C1C-387F-4E3D-A54F-CF1D913A6676}" name="ID_MODALIDADE" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{409E0C8E-C00D-45B9-8113-E86B37049A97}" name="MODALIDADE" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{9B83D5E8-C0D6-41D3-A5EB-27263A3A1DDA}" name="TIPO" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{D7FE0EEE-44EA-4C6B-B889-B4C030F1B758}" name=" DESCRICAO" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2AD56904-85CF-4C47-A092-1CC4D719D317}" name="tblCalendario" displayName="tblCalendario" ref="A1:G366" totalsRowShown="0" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2AD56904-85CF-4C47-A092-1CC4D719D317}" name="tblCalendario" displayName="tblCalendario" ref="A1:G366" totalsRowShown="0" dataDxfId="47">
   <autoFilter ref="A1:G366" xr:uid="{2AD56904-85CF-4C47-A092-1CC4D719D317}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F779E569-925E-439D-B1E1-8D86C934DF94}" name="DATA" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{9910EA8A-79F0-4CBA-B0EA-76C6A01D1DA2}" name="DIA_SEMANA" dataDxfId="48">
+    <tableColumn id="1" xr3:uid="{F779E569-925E-439D-B1E1-8D86C934DF94}" name="DATA" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{9910EA8A-79F0-4CBA-B0EA-76C6A01D1DA2}" name="DIA_SEMANA" dataDxfId="45">
       <calculatedColumnFormula>TEXT(A2,"dddd")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B5623804-AA40-4BA7-B2EB-75E1D43E1DDA}" name="MÊS" dataDxfId="47">
+    <tableColumn id="3" xr3:uid="{B5623804-AA40-4BA7-B2EB-75E1D43E1DDA}" name="MÊS" dataDxfId="44">
       <calculatedColumnFormula>TEXT(A2,"mmmm")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{353E7915-D743-4718-B4A3-CE0D53F4A516}" name="ANO" dataDxfId="46">
+    <tableColumn id="4" xr3:uid="{353E7915-D743-4718-B4A3-CE0D53F4A516}" name="ANO" dataDxfId="43">
       <calculatedColumnFormula>YEAR(A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{816AC587-9819-42DF-80FD-264F991CF8F3}" name="TIPO_DIA" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{7A6D793C-B684-4E23-A357-D584AE0AC6FD}" name="DESCRICAO" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{5B786348-03B6-441E-A7B1-194F3AA43107}" name="DIA_UTIL" dataDxfId="43">
+    <tableColumn id="5" xr3:uid="{816AC587-9819-42DF-80FD-264F991CF8F3}" name="TIPO_DIA" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{7A6D793C-B684-4E23-A357-D584AE0AC6FD}" name="DESCRICAO" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{5B786348-03B6-441E-A7B1-194F3AA43107}" name="DIA_UTIL" dataDxfId="40">
       <calculatedColumnFormula>IF(OR(E2="Feriado",E2="Recesso",B2="domingo",B2="sábado"),"NÃO","SIM")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1706,41 +1706,41 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10D39EA4-9F67-4E18-B764-60076E4485F8}" name="tblInstrutores" displayName="tblInstrutores" ref="A1:I14" totalsRowShown="0" headerRowDxfId="42" dataDxfId="40" headerRowBorderDxfId="41" tableBorderDxfId="39" totalsRowBorderDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10D39EA4-9F67-4E18-B764-60076E4485F8}" name="tblInstrutores" displayName="tblInstrutores" ref="A1:I14" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" headerRowBorderDxfId="38" tableBorderDxfId="36" totalsRowBorderDxfId="35">
   <autoFilter ref="A1:I14" xr:uid="{10D39EA4-9F67-4E18-B764-60076E4485F8}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G14">
     <sortCondition ref="B1:B14"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E0F79A67-2297-4B4A-A8E9-7102EE99B694}" name="ID" dataDxfId="37">
+    <tableColumn id="1" xr3:uid="{E0F79A67-2297-4B4A-A8E9-7102EE99B694}" name="ID" dataDxfId="34">
       <calculatedColumnFormula>IF(B2&lt;&gt;"",ROW()-1,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{532A9770-E647-4D50-B202-8BBE5806648D}" name="NOME_COMPLETO" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{DD24D10E-34AA-4D8E-B5F7-9B0E7D84B23A}" name="NOME_PADRONIZADO" dataDxfId="35">
+    <tableColumn id="2" xr3:uid="{532A9770-E647-4D50-B202-8BBE5806648D}" name="NOME_COMPLETO" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{DD24D10E-34AA-4D8E-B5F7-9B0E7D84B23A}" name="NOME_PADRONIZADO" dataDxfId="32">
       <calculatedColumnFormula>UPPER(B2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0DC783F1-8A1B-443E-A9AF-DB40A28DED0F}" name="STATUS" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{8E33C3CA-EB70-43F9-B178-A5FD7FB25151}" name="TELEFONE" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{6BB804C3-6D00-4CBA-AADC-80AA2AA5F0B3}" name="EMAIL" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{066724F8-E631-4356-AF06-A44B57F600FB}" name="CARGA_HORARIA_SEMANAL" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{18D3697E-D2C6-4E06-9624-B784D6581D8D}" name="HABILITADO_EAD" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{0523A053-C6F6-4529-94E2-81C8ABD9D627}" name="OBSERVAÇÃO" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{0DC783F1-8A1B-443E-A9AF-DB40A28DED0F}" name="STATUS" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{8E33C3CA-EB70-43F9-B178-A5FD7FB25151}" name="TELEFONE" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{6BB804C3-6D00-4CBA-AADC-80AA2AA5F0B3}" name="EMAIL" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{066724F8-E631-4356-AF06-A44B57F600FB}" name="CARGA_HORARIA_SEMANAL" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{18D3697E-D2C6-4E06-9624-B784D6581D8D}" name="HABILITADO_EAD" dataDxfId="27"/>
+    <tableColumn id="10" xr3:uid="{0523A053-C6F6-4529-94E2-81C8ABD9D627}" name="OBSERVAÇÃO" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DFA01504-D869-4496-AFB3-1B2D28A46752}" name="tblAmbientes" displayName="tblAmbientes" ref="A1:E17" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DFA01504-D869-4496-AFB3-1B2D28A46752}" name="tblAmbientes" displayName="tblAmbientes" ref="A1:E17" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="A1:E17" xr:uid="{DFA01504-D869-4496-AFB3-1B2D28A46752}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{4CC770AA-6DA6-4EFC-AAF1-5A329E637763}" name="ID" dataDxfId="26">
+    <tableColumn id="1" xr3:uid="{4CC770AA-6DA6-4EFC-AAF1-5A329E637763}" name="ID" dataDxfId="23">
       <calculatedColumnFormula>IF(B2&lt;&gt;"",ROW()-1,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B3952270-EACA-4683-9C35-CB58270B3617}" name="NOME_AMBIENTE" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{1B401582-0E5F-494F-8433-828BC136B12C}" name="TIPO" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{81780B59-8350-421A-B267-D808DA35B87C}" name="CAPACIDADE" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{7A3E5A22-F966-4BA3-A1AA-3C3AF64EA9D1}" name="VIRTUAL" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{B3952270-EACA-4683-9C35-CB58270B3617}" name="NOME_AMBIENTE" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{1B401582-0E5F-494F-8433-828BC136B12C}" name="TIPO" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{81780B59-8350-421A-B267-D808DA35B87C}" name="CAPACIDADE" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{7A3E5A22-F966-4BA3-A1AA-3C3AF64EA9D1}" name="VIRTUAL" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1750,14 +1750,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{27B64AF7-6011-40DE-B8EB-AFCA2AA948F7}" name="tblDisciplinas" displayName="tblDisciplinas" ref="A2:G29" totalsRowShown="0">
   <autoFilter ref="A2:G29" xr:uid="{27B64AF7-6011-40DE-B8EB-AFCA2AA948F7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EAB3743F-4C6C-47DC-9FAE-3B30927E6D25}" name="ID_DISCIPLINA" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{EAB3743F-4C6C-47DC-9FAE-3B30927E6D25}" name="ID_DISCIPLINA" dataDxfId="64">
       <calculatedColumnFormula>IF(E3&lt;&gt;"",ROW()-2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{AB44C0DC-4B9E-4D40-B9CB-D5B9E3AB1664}" name="ID_TURMA" dataDxfId="20">
+    <tableColumn id="7" xr3:uid="{AB44C0DC-4B9E-4D40-B9CB-D5B9E3AB1664}" name="ID_TURMA" dataDxfId="63">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblDisciplinas[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[ID_TURMA],"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{71F544AA-7A31-4153-B640-2C9D09A01400}" name="TURMA"/>
-    <tableColumn id="10" xr3:uid="{6CF7FD1A-08A6-4FC7-8349-E61A732E9B9A}" name="NOME_TURMA" dataDxfId="19">
+    <tableColumn id="10" xr3:uid="{6CF7FD1A-08A6-4FC7-8349-E61A732E9B9A}" name="NOME_TURMA" dataDxfId="62">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblDisciplinas[[#This Row],[TURMA]], tblTurmas[CODIGO_TURMA], tblTurmas[NOME_TURMA],"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{912B15BB-5B7F-4D54-B4D5-F1F5D64871C5}" name="NOME_DISCIPLINA"/>
@@ -2192,13 +2192,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B3" s="2">
         <f ca="1">TODAY()</f>
-        <v>46108</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="B15" s="4">
         <f>AVERAGEIFS(tblOcupacao[PERCENTUAL_OCUPACAO], tblOcupacao[ID_TURNO], 1)</f>
-        <v>0.77499999999999991</v>
+        <v>0.77976190476190477</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -3072,12 +3072,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="27" t="s">
@@ -12610,15 +12610,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
       <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -15149,90 +15149,142 @@
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" t="str">
+      <c r="B22" s="2">
+        <v>46111</v>
+      </c>
+      <c r="C22">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[ID_TURMA],"")</f>
-        <v/>
-      </c>
-      <c r="E22" t="str">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>194</v>
+      </c>
+      <c r="E22">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[DISCIPLINA]],tblDisciplinas[NOME_DISCIPLINA],tblDisciplinas[ID_DISCIPLINA],"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="40"/>
-      <c r="G22" t="str">
+        <v>2</v>
+      </c>
+      <c r="F22" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="G22">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[Nome do Instrutor]],tblInstrutores[NOME_COMPLETO],tblInstrutores[ID],"")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="H22" t="str">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[INSTRUTOR],"")</f>
-        <v/>
-      </c>
-      <c r="I22" t="str">
+        <v>Deilson dos Santos de Aquino</v>
+      </c>
+      <c r="I22">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[AMBIENTE]],tblAmbientes[NOME_AMBIENTE],tblAmbientes[ID],"")</f>
-        <v/>
-      </c>
-      <c r="K22" t="str">
+        <v>4</v>
+      </c>
+      <c r="J22" t="s">
+        <v>106</v>
+      </c>
+      <c r="K22">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],['#VALOR!]],tblTurnos[TURNO],tblTurnos[ID_TURNO],"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="L22" t="str">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[TURNO],"")</f>
-        <v/>
-      </c>
-      <c r="M22" t="str">
+        <v>MANHÃ</v>
+      </c>
+      <c r="M22">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[MODALIDADE]], tblModalidades[MODALIDADE], tblModalidades[ID_MODALIDADE],"")</f>
-        <v/>
-      </c>
-      <c r="O22" s="32"/>
-      <c r="P22" s="32"/>
-      <c r="Q22" s="33" t="e">
+        <v>1</v>
+      </c>
+      <c r="N22" t="s">
+        <v>18</v>
+      </c>
+      <c r="O22" s="32">
+        <v>0.375</v>
+      </c>
+      <c r="P22" s="32">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="Q22" s="33">
         <f>($P22-$O22)-_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[INTERVALO],"")</f>
-        <v>#VALUE!</v>
+        <v>0.23958333333333329</v>
+      </c>
+      <c r="R22">
+        <v>21</v>
+      </c>
+      <c r="S22" t="s">
+        <v>192</v>
+      </c>
+      <c r="T22" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" t="str">
+      <c r="B23" s="2">
+        <v>46108</v>
+      </c>
+      <c r="C23">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[ID_TURMA],"")</f>
-        <v/>
-      </c>
-      <c r="E23" t="str">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
+        <v>203</v>
+      </c>
+      <c r="E23">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[DISCIPLINA]],tblDisciplinas[NOME_DISCIPLINA],tblDisciplinas[ID_DISCIPLINA],"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="40"/>
-      <c r="G23" t="str">
+        <v>11</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>220</v>
+      </c>
+      <c r="G23">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[Nome do Instrutor]],tblInstrutores[NOME_COMPLETO],tblInstrutores[ID],"")</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="H23" t="str">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[INSTRUTOR],"")</f>
-        <v/>
-      </c>
-      <c r="I23" t="str">
+        <v>Raphael Barreto de Oliveira</v>
+      </c>
+      <c r="I23">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[AMBIENTE]],tblAmbientes[NOME_AMBIENTE],tblAmbientes[ID],"")</f>
-        <v/>
-      </c>
-      <c r="K23" t="str">
+        <v>4</v>
+      </c>
+      <c r="J23" t="s">
+        <v>106</v>
+      </c>
+      <c r="K23">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],['#VALOR!]],tblTurnos[TURNO],tblTurnos[ID_TURNO],"")</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="L23" t="str">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[TURNO],"")</f>
-        <v/>
-      </c>
-      <c r="M23" t="str">
+        <v>MANHÃ</v>
+      </c>
+      <c r="M23">
         <f>_xlfn.XLOOKUP(tblAlocacao[[#This Row],[MODALIDADE]], tblModalidades[MODALIDADE], tblModalidades[ID_MODALIDADE],"")</f>
-        <v/>
-      </c>
-      <c r="O23" s="32"/>
-      <c r="P23" s="32"/>
-      <c r="Q23" s="33" t="e">
+        <v>1</v>
+      </c>
+      <c r="N23" t="s">
+        <v>18</v>
+      </c>
+      <c r="O23" s="32">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="P23" s="32">
+        <v>0.5</v>
+      </c>
+      <c r="Q23" s="33">
         <f>($P23-$O23)-_xlfn.XLOOKUP(tblAlocacao[[#This Row],[TURMA]],tblTurmas[CODIGO_TURMA],tblTurmas[INTERVALO],"")</f>
-        <v>#VALUE!</v>
+        <v>0.15625000000000003</v>
+      </c>
+      <c r="R23">
+        <v>15</v>
+      </c>
+      <c r="S23" t="s">
+        <v>192</v>
+      </c>
+      <c r="T23" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.35">
@@ -27194,7 +27246,7 @@
         <v>24</v>
       </c>
       <c r="H2" s="35">
-        <f>$F2/$G2</f>
+        <f t="shared" ref="H2:H18" si="0">$F2/$G2</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="I2" t="str">
@@ -27230,7 +27282,7 @@
         <v>24</v>
       </c>
       <c r="H3" s="35">
-        <f>$F3/$G3</f>
+        <f t="shared" si="0"/>
         <v>0.91666666666666663</v>
       </c>
       <c r="I3" t="str">
@@ -27266,7 +27318,7 @@
         <v>24</v>
       </c>
       <c r="H4" s="35">
-        <f>$F4/$G4</f>
+        <f t="shared" si="0"/>
         <v>0.91666666666666663</v>
       </c>
       <c r="I4" t="str">
@@ -27302,7 +27354,7 @@
         <v>24</v>
       </c>
       <c r="H5" s="35">
-        <f>$F5/$G5</f>
+        <f t="shared" si="0"/>
         <v>0.91666666666666663</v>
       </c>
       <c r="I5" t="str">
@@ -27338,7 +27390,7 @@
         <v>24</v>
       </c>
       <c r="H6" s="35">
-        <f>$F6/$G6</f>
+        <f t="shared" si="0"/>
         <v>0.875</v>
       </c>
       <c r="I6" t="str">
@@ -27374,7 +27426,7 @@
         <v>24</v>
       </c>
       <c r="H7" s="35">
-        <f>$F7/$G7</f>
+        <f t="shared" si="0"/>
         <v>0.875</v>
       </c>
       <c r="I7" t="str">
@@ -27410,7 +27462,7 @@
         <v>24</v>
       </c>
       <c r="H8" s="35">
-        <f>$F8/$G8</f>
+        <f t="shared" si="0"/>
         <v>0.875</v>
       </c>
       <c r="I8" t="str">
@@ -27446,7 +27498,7 @@
         <v>24</v>
       </c>
       <c r="H9" s="35">
-        <f>$F9/$G9</f>
+        <f t="shared" si="0"/>
         <v>0.91666666666666663</v>
       </c>
       <c r="I9" t="str">
@@ -27482,7 +27534,7 @@
         <v>24</v>
       </c>
       <c r="H10" s="35">
-        <f>$F10/$G10</f>
+        <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
       <c r="I10" t="str">
@@ -27518,7 +27570,7 @@
         <v>24</v>
       </c>
       <c r="H11" s="35">
-        <f>$F11/$G11</f>
+        <f t="shared" si="0"/>
         <v>0.91666666666666663</v>
       </c>
       <c r="I11" t="str">
@@ -27554,7 +27606,7 @@
         <v>24</v>
       </c>
       <c r="H12" s="35">
-        <f>$F12/$G12</f>
+        <f t="shared" si="0"/>
         <v>0.91666666666666663</v>
       </c>
       <c r="I12" t="str">
@@ -27590,7 +27642,7 @@
         <v>24</v>
       </c>
       <c r="H13" s="35">
-        <f>$F13/$G13</f>
+        <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
       <c r="I13" t="str">
@@ -27626,7 +27678,7 @@
         <v>24</v>
       </c>
       <c r="H14" s="35">
-        <f>$F14/$G14</f>
+        <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
       <c r="I14" t="str">
@@ -27662,7 +27714,7 @@
         <v>24</v>
       </c>
       <c r="H15" s="35">
-        <f>$F15/$G15</f>
+        <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
       <c r="I15" t="str">
@@ -27698,7 +27750,7 @@
         <v>24</v>
       </c>
       <c r="H16" s="35">
-        <f>$F16/$G16</f>
+        <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
       <c r="I16" t="str">
@@ -27734,7 +27786,7 @@
         <v>24</v>
       </c>
       <c r="H17" s="35">
-        <f>$F17/$G17</f>
+        <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
       <c r="I17" t="str">
@@ -27770,7 +27822,7 @@
         <v>24</v>
       </c>
       <c r="H18" s="35">
-        <f>$F18/$G18</f>
+        <f t="shared" si="0"/>
         <v>0.625</v>
       </c>
       <c r="I18" t="str">
@@ -27806,7 +27858,7 @@
         <v>24</v>
       </c>
       <c r="H19" s="35">
-        <f t="shared" ref="H19:H21" si="0">$F19/$G19</f>
+        <f t="shared" ref="H19:H21" si="1">$F19/$G19</f>
         <v>0.625</v>
       </c>
       <c r="I19" t="str">
@@ -27842,7 +27894,7 @@
         <v>24</v>
       </c>
       <c r="H20" s="35">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.625</v>
       </c>
       <c r="I20" t="str">
@@ -27878,7 +27930,7 @@
         <v>24</v>
       </c>
       <c r="H21" s="35">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.625</v>
       </c>
       <c r="I21" t="str">
@@ -27890,22 +27942,39 @@
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="2"/>
-      <c r="B22" t="str">
-        <f>_xlfn.XLOOKUP(tblOcupacao[[#This Row],[AMBIENTE]],tblAmbientes[NOME_AMBIENTE],tblAmbientes[ID],"")</f>
-        <v/>
-      </c>
-      <c r="D22" t="str">
-        <f>_xlfn.XLOOKUP(tblOcupacao[[#This Row],[TURNO]],tblTurnos[TURNO],tblTurnos[ID_TURNO],"")</f>
-        <v/>
-      </c>
-      <c r="H22" s="35" t="e">
-        <f>$F22/$G22</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I22" t="e">
-        <f>IF(tblOcupacao[[#This Row],[PERCENTUAL_OCUPACAO]]&gt;0.75,"ALTA",IF(AND(tblOcupacao[[#This Row],[PERCENTUAL_OCUPACAO]]&lt;0.74,tblOcupacao[[#This Row],[PERCENTUAL_OCUPACAO]]&gt;0.5),"MÉDIO","BAIXO"))</f>
-        <v>#DIV/0!</v>
+      <c r="A22" s="2">
+        <v>46111</v>
+      </c>
+      <c r="B22">
+        <f>_xlfn.XLOOKUP(tblOcupacao[[#This Row],[AMBIENTE]],tblAmbientes[NOME_AMBIENTE],tblAmbientes[ID],"")</f>
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>106</v>
+      </c>
+      <c r="D22">
+        <f>_xlfn.XLOOKUP(tblOcupacao[[#This Row],[TURNO]],tblTurnos[TURNO],tblTurnos[ID_TURNO],"")</f>
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F22">
+        <v>21</v>
+      </c>
+      <c r="G22">
+        <v>24</v>
+      </c>
+      <c r="H22" s="35">
+        <f t="shared" ref="H22:H85" si="2">$F22/$G22</f>
+        <v>0.875</v>
+      </c>
+      <c r="I22" t="str">
+        <f>IF(tblOcupacao[[#This Row],[PERCENTUAL_OCUPACAO]]&gt;0.75,"ALTA",IF(AND(tblOcupacao[[#This Row],[PERCENTUAL_OCUPACAO]]&lt;0.74,tblOcupacao[[#This Row],[PERCENTUAL_OCUPACAO]]&gt;0.5),"MÉDIO","BAIXO"))</f>
+        <v>ALTA</v>
+      </c>
+      <c r="J22" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -27919,7 +27988,7 @@
         <v/>
       </c>
       <c r="H23" s="35" t="e">
-        <f>$F23/$G23</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I23" t="e">
@@ -27938,7 +28007,7 @@
         <v/>
       </c>
       <c r="H24" s="35" t="e">
-        <f>$F24/$G24</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I24" t="e">
@@ -27957,7 +28026,7 @@
         <v/>
       </c>
       <c r="H25" s="35" t="e">
-        <f>$F25/$G25</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I25" t="e">
@@ -27976,7 +28045,7 @@
         <v/>
       </c>
       <c r="H26" s="35" t="e">
-        <f>$F26/$G26</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I26" t="e">
@@ -27995,7 +28064,7 @@
         <v/>
       </c>
       <c r="H27" s="35" t="e">
-        <f>$F27/$G27</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I27" t="e">
@@ -28014,7 +28083,7 @@
         <v/>
       </c>
       <c r="H28" s="35" t="e">
-        <f>$F28/$G28</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I28" t="e">
@@ -28033,7 +28102,7 @@
         <v/>
       </c>
       <c r="H29" s="35" t="e">
-        <f>$F29/$G29</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I29" t="e">
@@ -28052,7 +28121,7 @@
         <v/>
       </c>
       <c r="H30" s="35" t="e">
-        <f>$F30/$G30</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I30" t="e">
@@ -28071,7 +28140,7 @@
         <v/>
       </c>
       <c r="H31" s="35" t="e">
-        <f>$F31/$G31</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I31" t="e">
@@ -28090,7 +28159,7 @@
         <v/>
       </c>
       <c r="H32" s="35" t="e">
-        <f>$F32/$G32</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I32" t="e">
@@ -28109,7 +28178,7 @@
         <v/>
       </c>
       <c r="H33" s="35" t="e">
-        <f>$F33/$G33</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I33" t="e">
@@ -28128,7 +28197,7 @@
         <v/>
       </c>
       <c r="H34" s="35" t="e">
-        <f>$F34/$G34</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I34" t="e">
@@ -28147,7 +28216,7 @@
         <v/>
       </c>
       <c r="H35" s="35" t="e">
-        <f>$F35/$G35</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I35" t="e">
@@ -28166,7 +28235,7 @@
         <v/>
       </c>
       <c r="H36" s="35" t="e">
-        <f>$F36/$G36</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I36" t="e">
@@ -28185,7 +28254,7 @@
         <v/>
       </c>
       <c r="H37" s="35" t="e">
-        <f>$F37/$G37</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I37" t="e">
@@ -28204,7 +28273,7 @@
         <v/>
       </c>
       <c r="H38" s="35" t="e">
-        <f>$F38/$G38</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I38" t="e">
@@ -28223,7 +28292,7 @@
         <v/>
       </c>
       <c r="H39" s="35" t="e">
-        <f>$F39/$G39</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I39" t="e">
@@ -28242,7 +28311,7 @@
         <v/>
       </c>
       <c r="H40" s="35" t="e">
-        <f>$F40/$G40</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I40" t="e">
@@ -28261,7 +28330,7 @@
         <v/>
       </c>
       <c r="H41" s="35" t="e">
-        <f>$F41/$G41</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I41" t="e">
@@ -28280,7 +28349,7 @@
         <v/>
       </c>
       <c r="H42" s="35" t="e">
-        <f>$F42/$G42</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I42" t="e">
@@ -28299,7 +28368,7 @@
         <v/>
       </c>
       <c r="H43" s="35" t="e">
-        <f>$F43/$G43</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I43" t="e">
@@ -28318,7 +28387,7 @@
         <v/>
       </c>
       <c r="H44" s="35" t="e">
-        <f>$F44/$G44</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I44" t="e">
@@ -28337,7 +28406,7 @@
         <v/>
       </c>
       <c r="H45" s="35" t="e">
-        <f>$F45/$G45</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I45" t="e">
@@ -28356,7 +28425,7 @@
         <v/>
       </c>
       <c r="H46" s="35" t="e">
-        <f>$F46/$G46</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I46" t="e">
@@ -28375,7 +28444,7 @@
         <v/>
       </c>
       <c r="H47" s="35" t="e">
-        <f>$F47/$G47</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I47" t="e">
@@ -28394,7 +28463,7 @@
         <v/>
       </c>
       <c r="H48" s="35" t="e">
-        <f>$F48/$G48</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I48" t="e">
@@ -28413,7 +28482,7 @@
         <v/>
       </c>
       <c r="H49" s="35" t="e">
-        <f>$F49/$G49</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I49" t="e">
@@ -28432,7 +28501,7 @@
         <v/>
       </c>
       <c r="H50" s="35" t="e">
-        <f>$F50/$G50</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I50" t="e">
@@ -28451,7 +28520,7 @@
         <v/>
       </c>
       <c r="H51" s="35" t="e">
-        <f>$F51/$G51</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I51" t="e">
@@ -28470,7 +28539,7 @@
         <v/>
       </c>
       <c r="H52" s="35" t="e">
-        <f>$F52/$G52</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I52" t="e">
@@ -28489,7 +28558,7 @@
         <v/>
       </c>
       <c r="H53" s="35" t="e">
-        <f>$F53/$G53</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I53" t="e">
@@ -28508,7 +28577,7 @@
         <v/>
       </c>
       <c r="H54" s="35" t="e">
-        <f>$F54/$G54</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I54" t="e">
@@ -28527,7 +28596,7 @@
         <v/>
       </c>
       <c r="H55" s="35" t="e">
-        <f>$F55/$G55</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I55" t="e">
@@ -28546,7 +28615,7 @@
         <v/>
       </c>
       <c r="H56" s="35" t="e">
-        <f>$F56/$G56</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I56" t="e">
@@ -28565,7 +28634,7 @@
         <v/>
       </c>
       <c r="H57" s="35" t="e">
-        <f>$F57/$G57</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I57" t="e">
@@ -28584,7 +28653,7 @@
         <v/>
       </c>
       <c r="H58" s="35" t="e">
-        <f>$F58/$G58</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I58" t="e">
@@ -28603,7 +28672,7 @@
         <v/>
       </c>
       <c r="H59" s="35" t="e">
-        <f>$F59/$G59</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I59" t="e">
@@ -28622,7 +28691,7 @@
         <v/>
       </c>
       <c r="H60" s="35" t="e">
-        <f>$F60/$G60</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I60" t="e">
@@ -28641,7 +28710,7 @@
         <v/>
       </c>
       <c r="H61" s="35" t="e">
-        <f>$F61/$G61</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I61" t="e">
@@ -28660,7 +28729,7 @@
         <v/>
       </c>
       <c r="H62" s="35" t="e">
-        <f>$F62/$G62</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I62" t="e">
@@ -28679,7 +28748,7 @@
         <v/>
       </c>
       <c r="H63" s="35" t="e">
-        <f>$F63/$G63</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I63" t="e">
@@ -28698,7 +28767,7 @@
         <v/>
       </c>
       <c r="H64" s="35" t="e">
-        <f>$F64/$G64</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I64" t="e">
@@ -28717,7 +28786,7 @@
         <v/>
       </c>
       <c r="H65" s="35" t="e">
-        <f>$F65/$G65</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I65" t="e">
@@ -28736,7 +28805,7 @@
         <v/>
       </c>
       <c r="H66" s="35" t="e">
-        <f>$F66/$G66</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I66" t="e">
@@ -28755,7 +28824,7 @@
         <v/>
       </c>
       <c r="H67" s="35" t="e">
-        <f>$F67/$G67</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I67" t="e">
@@ -28774,7 +28843,7 @@
         <v/>
       </c>
       <c r="H68" s="35" t="e">
-        <f>$F68/$G68</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I68" t="e">
@@ -28793,7 +28862,7 @@
         <v/>
       </c>
       <c r="H69" s="35" t="e">
-        <f>$F69/$G69</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I69" t="e">
@@ -28812,7 +28881,7 @@
         <v/>
       </c>
       <c r="H70" s="35" t="e">
-        <f>$F70/$G70</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I70" t="e">
@@ -28831,7 +28900,7 @@
         <v/>
       </c>
       <c r="H71" s="35" t="e">
-        <f>$F71/$G71</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I71" t="e">
@@ -28850,7 +28919,7 @@
         <v/>
       </c>
       <c r="H72" s="35" t="e">
-        <f>$F72/$G72</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I72" t="e">
@@ -28869,7 +28938,7 @@
         <v/>
       </c>
       <c r="H73" s="35" t="e">
-        <f>$F73/$G73</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I73" t="e">
@@ -28888,7 +28957,7 @@
         <v/>
       </c>
       <c r="H74" s="35" t="e">
-        <f>$F74/$G74</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I74" t="e">
@@ -28907,7 +28976,7 @@
         <v/>
       </c>
       <c r="H75" s="35" t="e">
-        <f>$F75/$G75</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I75" t="e">
@@ -28926,7 +28995,7 @@
         <v/>
       </c>
       <c r="H76" s="35" t="e">
-        <f>$F76/$G76</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I76" t="e">
@@ -28945,7 +29014,7 @@
         <v/>
       </c>
       <c r="H77" s="35" t="e">
-        <f>$F77/$G77</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I77" t="e">
@@ -28964,7 +29033,7 @@
         <v/>
       </c>
       <c r="H78" s="35" t="e">
-        <f>$F78/$G78</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I78" t="e">
@@ -28983,7 +29052,7 @@
         <v/>
       </c>
       <c r="H79" s="35" t="e">
-        <f>$F79/$G79</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I79" t="e">
@@ -29002,7 +29071,7 @@
         <v/>
       </c>
       <c r="H80" s="35" t="e">
-        <f>$F80/$G80</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I80" t="e">
@@ -29021,7 +29090,7 @@
         <v/>
       </c>
       <c r="H81" s="35" t="e">
-        <f>$F81/$G81</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I81" t="e">
@@ -29040,7 +29109,7 @@
         <v/>
       </c>
       <c r="H82" s="35" t="e">
-        <f>$F82/$G82</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I82" t="e">
@@ -29059,7 +29128,7 @@
         <v/>
       </c>
       <c r="H83" s="35" t="e">
-        <f>$F83/$G83</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I83" t="e">
@@ -29078,7 +29147,7 @@
         <v/>
       </c>
       <c r="H84" s="35" t="e">
-        <f>$F84/$G84</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I84" t="e">
@@ -29097,7 +29166,7 @@
         <v/>
       </c>
       <c r="H85" s="35" t="e">
-        <f>$F85/$G85</f>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I85" t="e">
@@ -29116,7 +29185,7 @@
         <v/>
       </c>
       <c r="H86" s="35" t="e">
-        <f>$F86/$G86</f>
+        <f t="shared" ref="H86:H149" si="3">$F86/$G86</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I86" t="e">
@@ -29135,7 +29204,7 @@
         <v/>
       </c>
       <c r="H87" s="35" t="e">
-        <f>$F87/$G87</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I87" t="e">
@@ -29154,7 +29223,7 @@
         <v/>
       </c>
       <c r="H88" s="35" t="e">
-        <f>$F88/$G88</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I88" t="e">
@@ -29173,7 +29242,7 @@
         <v/>
       </c>
       <c r="H89" s="35" t="e">
-        <f>$F89/$G89</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I89" t="e">
@@ -29192,7 +29261,7 @@
         <v/>
       </c>
       <c r="H90" s="35" t="e">
-        <f>$F90/$G90</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I90" t="e">
@@ -29211,7 +29280,7 @@
         <v/>
       </c>
       <c r="H91" s="35" t="e">
-        <f>$F91/$G91</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I91" t="e">
@@ -29230,7 +29299,7 @@
         <v/>
       </c>
       <c r="H92" s="35" t="e">
-        <f>$F92/$G92</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I92" t="e">
@@ -29249,7 +29318,7 @@
         <v/>
       </c>
       <c r="H93" s="35" t="e">
-        <f>$F93/$G93</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I93" t="e">
@@ -29268,7 +29337,7 @@
         <v/>
       </c>
       <c r="H94" s="35" t="e">
-        <f>$F94/$G94</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I94" t="e">
@@ -29287,7 +29356,7 @@
         <v/>
       </c>
       <c r="H95" s="35" t="e">
-        <f>$F95/$G95</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I95" t="e">
@@ -29306,7 +29375,7 @@
         <v/>
       </c>
       <c r="H96" s="35" t="e">
-        <f>$F96/$G96</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I96" t="e">
@@ -29325,7 +29394,7 @@
         <v/>
       </c>
       <c r="H97" s="35" t="e">
-        <f>$F97/$G97</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I97" t="e">
@@ -29344,7 +29413,7 @@
         <v/>
       </c>
       <c r="H98" s="35" t="e">
-        <f>$F98/$G98</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I98" t="e">
@@ -29363,7 +29432,7 @@
         <v/>
       </c>
       <c r="H99" s="35" t="e">
-        <f>$F99/$G99</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I99" t="e">
@@ -29382,7 +29451,7 @@
         <v/>
       </c>
       <c r="H100" s="35" t="e">
-        <f>$F100/$G100</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I100" t="e">
@@ -29401,7 +29470,7 @@
         <v/>
       </c>
       <c r="H101" s="35" t="e">
-        <f>$F101/$G101</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I101" t="e">
@@ -29420,7 +29489,7 @@
         <v/>
       </c>
       <c r="H102" s="35" t="e">
-        <f>$F102/$G102</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I102" t="e">
@@ -29439,7 +29508,7 @@
         <v/>
       </c>
       <c r="H103" s="35" t="e">
-        <f>$F103/$G103</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I103" t="e">
@@ -29458,7 +29527,7 @@
         <v/>
       </c>
       <c r="H104" s="35" t="e">
-        <f>$F104/$G104</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I104" t="e">
@@ -29477,7 +29546,7 @@
         <v/>
       </c>
       <c r="H105" s="35" t="e">
-        <f>$F105/$G105</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I105" t="e">
@@ -29496,7 +29565,7 @@
         <v/>
       </c>
       <c r="H106" s="35" t="e">
-        <f>$F106/$G106</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I106" t="e">
@@ -29515,7 +29584,7 @@
         <v/>
       </c>
       <c r="H107" s="35" t="e">
-        <f>$F107/$G107</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I107" t="e">
@@ -29534,7 +29603,7 @@
         <v/>
       </c>
       <c r="H108" s="35" t="e">
-        <f>$F108/$G108</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I108" t="e">
@@ -29553,7 +29622,7 @@
         <v/>
       </c>
       <c r="H109" s="35" t="e">
-        <f>$F109/$G109</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I109" t="e">
@@ -29572,7 +29641,7 @@
         <v/>
       </c>
       <c r="H110" s="35" t="e">
-        <f>$F110/$G110</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I110" t="e">
@@ -29591,7 +29660,7 @@
         <v/>
       </c>
       <c r="H111" s="35" t="e">
-        <f>$F111/$G111</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I111" t="e">
@@ -29610,7 +29679,7 @@
         <v/>
       </c>
       <c r="H112" s="35" t="e">
-        <f>$F112/$G112</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I112" t="e">
@@ -29629,7 +29698,7 @@
         <v/>
       </c>
       <c r="H113" s="35" t="e">
-        <f>$F113/$G113</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I113" t="e">
@@ -29648,7 +29717,7 @@
         <v/>
       </c>
       <c r="H114" s="35" t="e">
-        <f>$F114/$G114</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I114" t="e">
@@ -29667,7 +29736,7 @@
         <v/>
       </c>
       <c r="H115" s="35" t="e">
-        <f>$F115/$G115</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I115" t="e">
@@ -29686,7 +29755,7 @@
         <v/>
       </c>
       <c r="H116" s="35" t="e">
-        <f>$F116/$G116</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I116" t="e">
@@ -29705,7 +29774,7 @@
         <v/>
       </c>
       <c r="H117" s="35" t="e">
-        <f>$F117/$G117</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I117" t="e">
@@ -29724,7 +29793,7 @@
         <v/>
       </c>
       <c r="H118" s="35" t="e">
-        <f>$F118/$G118</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I118" t="e">
@@ -29743,7 +29812,7 @@
         <v/>
       </c>
       <c r="H119" s="35" t="e">
-        <f>$F119/$G119</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I119" t="e">
@@ -29762,7 +29831,7 @@
         <v/>
       </c>
       <c r="H120" s="35" t="e">
-        <f>$F120/$G120</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I120" t="e">
@@ -29781,7 +29850,7 @@
         <v/>
       </c>
       <c r="H121" s="35" t="e">
-        <f>$F121/$G121</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I121" t="e">
@@ -29800,7 +29869,7 @@
         <v/>
       </c>
       <c r="H122" s="35" t="e">
-        <f>$F122/$G122</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I122" t="e">
@@ -29819,7 +29888,7 @@
         <v/>
       </c>
       <c r="H123" s="35" t="e">
-        <f>$F123/$G123</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I123" t="e">
@@ -29838,7 +29907,7 @@
         <v/>
       </c>
       <c r="H124" s="35" t="e">
-        <f>$F124/$G124</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I124" t="e">
@@ -29857,7 +29926,7 @@
         <v/>
       </c>
       <c r="H125" s="35" t="e">
-        <f>$F125/$G125</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I125" t="e">
@@ -29876,7 +29945,7 @@
         <v/>
       </c>
       <c r="H126" s="35" t="e">
-        <f>$F126/$G126</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I126" t="e">
@@ -29895,7 +29964,7 @@
         <v/>
       </c>
       <c r="H127" s="35" t="e">
-        <f>$F127/$G127</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I127" t="e">
@@ -29914,7 +29983,7 @@
         <v/>
       </c>
       <c r="H128" s="35" t="e">
-        <f>$F128/$G128</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I128" t="e">
@@ -29933,7 +30002,7 @@
         <v/>
       </c>
       <c r="H129" s="35" t="e">
-        <f>$F129/$G129</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I129" t="e">
@@ -29952,7 +30021,7 @@
         <v/>
       </c>
       <c r="H130" s="35" t="e">
-        <f>$F130/$G130</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I130" t="e">
@@ -29971,7 +30040,7 @@
         <v/>
       </c>
       <c r="H131" s="35" t="e">
-        <f>$F131/$G131</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I131" t="e">
@@ -29990,7 +30059,7 @@
         <v/>
       </c>
       <c r="H132" s="35" t="e">
-        <f>$F132/$G132</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I132" t="e">
@@ -30009,7 +30078,7 @@
         <v/>
       </c>
       <c r="H133" s="35" t="e">
-        <f>$F133/$G133</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I133" t="e">
@@ -30028,7 +30097,7 @@
         <v/>
       </c>
       <c r="H134" s="35" t="e">
-        <f>$F134/$G134</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I134" t="e">
@@ -30047,7 +30116,7 @@
         <v/>
       </c>
       <c r="H135" s="35" t="e">
-        <f>$F135/$G135</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I135" t="e">
@@ -30066,7 +30135,7 @@
         <v/>
       </c>
       <c r="H136" s="35" t="e">
-        <f>$F136/$G136</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I136" t="e">
@@ -30085,7 +30154,7 @@
         <v/>
       </c>
       <c r="H137" s="35" t="e">
-        <f>$F137/$G137</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I137" t="e">
@@ -30104,7 +30173,7 @@
         <v/>
       </c>
       <c r="H138" s="35" t="e">
-        <f>$F138/$G138</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I138" t="e">
@@ -30123,7 +30192,7 @@
         <v/>
       </c>
       <c r="H139" s="35" t="e">
-        <f>$F139/$G139</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I139" t="e">
@@ -30142,7 +30211,7 @@
         <v/>
       </c>
       <c r="H140" s="35" t="e">
-        <f>$F140/$G140</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I140" t="e">
@@ -30161,7 +30230,7 @@
         <v/>
       </c>
       <c r="H141" s="35" t="e">
-        <f>$F141/$G141</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I141" t="e">
@@ -30180,7 +30249,7 @@
         <v/>
       </c>
       <c r="H142" s="35" t="e">
-        <f>$F142/$G142</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I142" t="e">
@@ -30199,7 +30268,7 @@
         <v/>
       </c>
       <c r="H143" s="35" t="e">
-        <f>$F143/$G143</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I143" t="e">
@@ -30218,7 +30287,7 @@
         <v/>
       </c>
       <c r="H144" s="35" t="e">
-        <f>$F144/$G144</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I144" t="e">
@@ -30237,7 +30306,7 @@
         <v/>
       </c>
       <c r="H145" s="35" t="e">
-        <f>$F145/$G145</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I145" t="e">
@@ -30256,7 +30325,7 @@
         <v/>
       </c>
       <c r="H146" s="35" t="e">
-        <f>$F146/$G146</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I146" t="e">
@@ -30275,7 +30344,7 @@
         <v/>
       </c>
       <c r="H147" s="35" t="e">
-        <f>$F147/$G147</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I147" t="e">
@@ -30294,7 +30363,7 @@
         <v/>
       </c>
       <c r="H148" s="35" t="e">
-        <f>$F148/$G148</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I148" t="e">
@@ -30313,7 +30382,7 @@
         <v/>
       </c>
       <c r="H149" s="35" t="e">
-        <f>$F149/$G149</f>
+        <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I149" t="e">
@@ -30332,7 +30401,7 @@
         <v/>
       </c>
       <c r="H150" s="35" t="e">
-        <f>$F150/$G150</f>
+        <f t="shared" ref="H150:H213" si="4">$F150/$G150</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I150" t="e">
@@ -30351,7 +30420,7 @@
         <v/>
       </c>
       <c r="H151" s="35" t="e">
-        <f>$F151/$G151</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I151" t="e">
@@ -30370,7 +30439,7 @@
         <v/>
       </c>
       <c r="H152" s="35" t="e">
-        <f>$F152/$G152</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I152" t="e">
@@ -30389,7 +30458,7 @@
         <v/>
       </c>
       <c r="H153" s="35" t="e">
-        <f>$F153/$G153</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I153" t="e">
@@ -30408,7 +30477,7 @@
         <v/>
       </c>
       <c r="H154" s="35" t="e">
-        <f>$F154/$G154</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I154" t="e">
@@ -30427,7 +30496,7 @@
         <v/>
       </c>
       <c r="H155" s="35" t="e">
-        <f>$F155/$G155</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I155" t="e">
@@ -30446,7 +30515,7 @@
         <v/>
       </c>
       <c r="H156" s="35" t="e">
-        <f>$F156/$G156</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I156" t="e">
@@ -30465,7 +30534,7 @@
         <v/>
       </c>
       <c r="H157" s="35" t="e">
-        <f>$F157/$G157</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I157" t="e">
@@ -30484,7 +30553,7 @@
         <v/>
       </c>
       <c r="H158" s="35" t="e">
-        <f>$F158/$G158</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I158" t="e">
@@ -30503,7 +30572,7 @@
         <v/>
       </c>
       <c r="H159" s="35" t="e">
-        <f>$F159/$G159</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I159" t="e">
@@ -30522,7 +30591,7 @@
         <v/>
       </c>
       <c r="H160" s="35" t="e">
-        <f>$F160/$G160</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I160" t="e">
@@ -30541,7 +30610,7 @@
         <v/>
       </c>
       <c r="H161" s="35" t="e">
-        <f>$F161/$G161</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I161" t="e">
@@ -30560,7 +30629,7 @@
         <v/>
       </c>
       <c r="H162" s="35" t="e">
-        <f>$F162/$G162</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I162" t="e">
@@ -30579,7 +30648,7 @@
         <v/>
       </c>
       <c r="H163" s="35" t="e">
-        <f>$F163/$G163</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I163" t="e">
@@ -30598,7 +30667,7 @@
         <v/>
       </c>
       <c r="H164" s="35" t="e">
-        <f>$F164/$G164</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I164" t="e">
@@ -30617,7 +30686,7 @@
         <v/>
       </c>
       <c r="H165" s="35" t="e">
-        <f>$F165/$G165</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I165" t="e">
@@ -30636,7 +30705,7 @@
         <v/>
       </c>
       <c r="H166" s="35" t="e">
-        <f>$F166/$G166</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I166" t="e">
@@ -30655,7 +30724,7 @@
         <v/>
       </c>
       <c r="H167" s="35" t="e">
-        <f>$F167/$G167</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I167" t="e">
@@ -30674,7 +30743,7 @@
         <v/>
       </c>
       <c r="H168" s="35" t="e">
-        <f>$F168/$G168</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I168" t="e">
@@ -30693,7 +30762,7 @@
         <v/>
       </c>
       <c r="H169" s="35" t="e">
-        <f>$F169/$G169</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I169" t="e">
@@ -30712,7 +30781,7 @@
         <v/>
       </c>
       <c r="H170" s="35" t="e">
-        <f>$F170/$G170</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I170" t="e">
@@ -30731,7 +30800,7 @@
         <v/>
       </c>
       <c r="H171" s="35" t="e">
-        <f>$F171/$G171</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I171" t="e">
@@ -30750,7 +30819,7 @@
         <v/>
       </c>
       <c r="H172" s="35" t="e">
-        <f>$F172/$G172</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I172" t="e">
@@ -30769,7 +30838,7 @@
         <v/>
       </c>
       <c r="H173" s="35" t="e">
-        <f>$F173/$G173</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I173" t="e">
@@ -30788,7 +30857,7 @@
         <v/>
       </c>
       <c r="H174" s="35" t="e">
-        <f>$F174/$G174</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I174" t="e">
@@ -30807,7 +30876,7 @@
         <v/>
       </c>
       <c r="H175" s="35" t="e">
-        <f>$F175/$G175</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I175" t="e">
@@ -30826,7 +30895,7 @@
         <v/>
       </c>
       <c r="H176" s="35" t="e">
-        <f>$F176/$G176</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I176" t="e">
@@ -30845,7 +30914,7 @@
         <v/>
       </c>
       <c r="H177" s="35" t="e">
-        <f>$F177/$G177</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I177" t="e">
@@ -30864,7 +30933,7 @@
         <v/>
       </c>
       <c r="H178" s="35" t="e">
-        <f>$F178/$G178</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I178" t="e">
@@ -30883,7 +30952,7 @@
         <v/>
       </c>
       <c r="H179" s="35" t="e">
-        <f>$F179/$G179</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I179" t="e">
@@ -30902,7 +30971,7 @@
         <v/>
       </c>
       <c r="H180" s="35" t="e">
-        <f>$F180/$G180</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I180" t="e">
@@ -30921,7 +30990,7 @@
         <v/>
       </c>
       <c r="H181" s="35" t="e">
-        <f>$F181/$G181</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I181" t="e">
@@ -30940,7 +31009,7 @@
         <v/>
       </c>
       <c r="H182" s="35" t="e">
-        <f>$F182/$G182</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I182" t="e">
@@ -30959,7 +31028,7 @@
         <v/>
       </c>
       <c r="H183" s="35" t="e">
-        <f>$F183/$G183</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I183" t="e">
@@ -30978,7 +31047,7 @@
         <v/>
       </c>
       <c r="H184" s="35" t="e">
-        <f>$F184/$G184</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I184" t="e">
@@ -30997,7 +31066,7 @@
         <v/>
       </c>
       <c r="H185" s="35" t="e">
-        <f>$F185/$G185</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I185" t="e">
@@ -31016,7 +31085,7 @@
         <v/>
       </c>
       <c r="H186" s="35" t="e">
-        <f>$F186/$G186</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I186" t="e">
@@ -31035,7 +31104,7 @@
         <v/>
       </c>
       <c r="H187" s="35" t="e">
-        <f>$F187/$G187</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I187" t="e">
@@ -31054,7 +31123,7 @@
         <v/>
       </c>
       <c r="H188" s="35" t="e">
-        <f>$F188/$G188</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I188" t="e">
@@ -31073,7 +31142,7 @@
         <v/>
       </c>
       <c r="H189" s="35" t="e">
-        <f>$F189/$G189</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I189" t="e">
@@ -31092,7 +31161,7 @@
         <v/>
       </c>
       <c r="H190" s="35" t="e">
-        <f>$F190/$G190</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I190" t="e">
@@ -31111,7 +31180,7 @@
         <v/>
       </c>
       <c r="H191" s="35" t="e">
-        <f>$F191/$G191</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I191" t="e">
@@ -31130,7 +31199,7 @@
         <v/>
       </c>
       <c r="H192" s="35" t="e">
-        <f>$F192/$G192</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I192" t="e">
@@ -31149,7 +31218,7 @@
         <v/>
       </c>
       <c r="H193" s="35" t="e">
-        <f>$F193/$G193</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I193" t="e">
@@ -31168,7 +31237,7 @@
         <v/>
       </c>
       <c r="H194" s="35" t="e">
-        <f>$F194/$G194</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I194" t="e">
@@ -31187,7 +31256,7 @@
         <v/>
       </c>
       <c r="H195" s="35" t="e">
-        <f>$F195/$G195</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I195" t="e">
@@ -31206,7 +31275,7 @@
         <v/>
       </c>
       <c r="H196" s="35" t="e">
-        <f>$F196/$G196</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I196" t="e">
@@ -31225,7 +31294,7 @@
         <v/>
       </c>
       <c r="H197" s="35" t="e">
-        <f>$F197/$G197</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I197" t="e">
@@ -31244,7 +31313,7 @@
         <v/>
       </c>
       <c r="H198" s="35" t="e">
-        <f>$F198/$G198</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I198" t="e">
@@ -31263,7 +31332,7 @@
         <v/>
       </c>
       <c r="H199" s="35" t="e">
-        <f>$F199/$G199</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I199" t="e">
@@ -31282,7 +31351,7 @@
         <v/>
       </c>
       <c r="H200" s="35" t="e">
-        <f>$F200/$G200</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I200" t="e">
@@ -31301,7 +31370,7 @@
         <v/>
       </c>
       <c r="H201" s="35" t="e">
-        <f>$F201/$G201</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I201" t="e">
@@ -31320,7 +31389,7 @@
         <v/>
       </c>
       <c r="H202" s="35" t="e">
-        <f>$F202/$G202</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I202" t="e">
@@ -31339,7 +31408,7 @@
         <v/>
       </c>
       <c r="H203" s="35" t="e">
-        <f>$F203/$G203</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I203" t="e">
@@ -31358,7 +31427,7 @@
         <v/>
       </c>
       <c r="H204" s="35" t="e">
-        <f>$F204/$G204</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I204" t="e">
@@ -31377,7 +31446,7 @@
         <v/>
       </c>
       <c r="H205" s="35" t="e">
-        <f>$F205/$G205</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I205" t="e">
@@ -31396,7 +31465,7 @@
         <v/>
       </c>
       <c r="H206" s="35" t="e">
-        <f>$F206/$G206</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I206" t="e">
@@ -31415,7 +31484,7 @@
         <v/>
       </c>
       <c r="H207" s="35" t="e">
-        <f>$F207/$G207</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I207" t="e">
@@ -31434,7 +31503,7 @@
         <v/>
       </c>
       <c r="H208" s="35" t="e">
-        <f>$F208/$G208</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I208" t="e">
@@ -31453,7 +31522,7 @@
         <v/>
       </c>
       <c r="H209" s="35" t="e">
-        <f>$F209/$G209</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I209" t="e">
@@ -31472,7 +31541,7 @@
         <v/>
       </c>
       <c r="H210" s="35" t="e">
-        <f>$F210/$G210</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I210" t="e">
@@ -31491,7 +31560,7 @@
         <v/>
       </c>
       <c r="H211" s="35" t="e">
-        <f>$F211/$G211</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I211" t="e">
@@ -31510,7 +31579,7 @@
         <v/>
       </c>
       <c r="H212" s="35" t="e">
-        <f>$F212/$G212</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I212" t="e">
@@ -31529,7 +31598,7 @@
         <v/>
       </c>
       <c r="H213" s="35" t="e">
-        <f>$F213/$G213</f>
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I213" t="e">
@@ -31548,7 +31617,7 @@
         <v/>
       </c>
       <c r="H214" s="35" t="e">
-        <f>$F214/$G214</f>
+        <f t="shared" ref="H214:H277" si="5">$F214/$G214</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I214" t="e">
@@ -31567,7 +31636,7 @@
         <v/>
       </c>
       <c r="H215" s="35" t="e">
-        <f>$F215/$G215</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I215" t="e">
@@ -31586,7 +31655,7 @@
         <v/>
       </c>
       <c r="H216" s="35" t="e">
-        <f>$F216/$G216</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I216" t="e">
@@ -31605,7 +31674,7 @@
         <v/>
       </c>
       <c r="H217" s="35" t="e">
-        <f>$F217/$G217</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I217" t="e">
@@ -31624,7 +31693,7 @@
         <v/>
       </c>
       <c r="H218" s="35" t="e">
-        <f>$F218/$G218</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I218" t="e">
@@ -31643,7 +31712,7 @@
         <v/>
       </c>
       <c r="H219" s="35" t="e">
-        <f>$F219/$G219</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I219" t="e">
@@ -31662,7 +31731,7 @@
         <v/>
       </c>
       <c r="H220" s="35" t="e">
-        <f>$F220/$G220</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I220" t="e">
@@ -31681,7 +31750,7 @@
         <v/>
       </c>
       <c r="H221" s="35" t="e">
-        <f>$F221/$G221</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I221" t="e">
@@ -31700,7 +31769,7 @@
         <v/>
       </c>
       <c r="H222" s="35" t="e">
-        <f>$F222/$G222</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I222" t="e">
@@ -31719,7 +31788,7 @@
         <v/>
       </c>
       <c r="H223" s="35" t="e">
-        <f>$F223/$G223</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I223" t="e">
@@ -31738,7 +31807,7 @@
         <v/>
       </c>
       <c r="H224" s="35" t="e">
-        <f>$F224/$G224</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I224" t="e">
@@ -31757,7 +31826,7 @@
         <v/>
       </c>
       <c r="H225" s="35" t="e">
-        <f>$F225/$G225</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I225" t="e">
@@ -31776,7 +31845,7 @@
         <v/>
       </c>
       <c r="H226" s="35" t="e">
-        <f>$F226/$G226</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I226" t="e">
@@ -31795,7 +31864,7 @@
         <v/>
       </c>
       <c r="H227" s="35" t="e">
-        <f>$F227/$G227</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I227" t="e">
@@ -31814,7 +31883,7 @@
         <v/>
       </c>
       <c r="H228" s="35" t="e">
-        <f>$F228/$G228</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I228" t="e">
@@ -31833,7 +31902,7 @@
         <v/>
       </c>
       <c r="H229" s="35" t="e">
-        <f>$F229/$G229</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I229" t="e">
@@ -31852,7 +31921,7 @@
         <v/>
       </c>
       <c r="H230" s="35" t="e">
-        <f>$F230/$G230</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I230" t="e">
@@ -31871,7 +31940,7 @@
         <v/>
       </c>
       <c r="H231" s="35" t="e">
-        <f>$F231/$G231</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I231" t="e">
@@ -31890,7 +31959,7 @@
         <v/>
       </c>
       <c r="H232" s="35" t="e">
-        <f>$F232/$G232</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I232" t="e">
@@ -31909,7 +31978,7 @@
         <v/>
       </c>
       <c r="H233" s="35" t="e">
-        <f>$F233/$G233</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I233" t="e">
@@ -31928,7 +31997,7 @@
         <v/>
       </c>
       <c r="H234" s="35" t="e">
-        <f>$F234/$G234</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I234" t="e">
@@ -31947,7 +32016,7 @@
         <v/>
       </c>
       <c r="H235" s="35" t="e">
-        <f>$F235/$G235</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I235" t="e">
@@ -31966,7 +32035,7 @@
         <v/>
       </c>
       <c r="H236" s="35" t="e">
-        <f>$F236/$G236</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I236" t="e">
@@ -31985,7 +32054,7 @@
         <v/>
       </c>
       <c r="H237" s="35" t="e">
-        <f>$F237/$G237</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I237" t="e">
@@ -32004,7 +32073,7 @@
         <v/>
       </c>
       <c r="H238" s="35" t="e">
-        <f>$F238/$G238</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I238" t="e">
@@ -32023,7 +32092,7 @@
         <v/>
       </c>
       <c r="H239" s="35" t="e">
-        <f>$F239/$G239</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I239" t="e">
@@ -32042,7 +32111,7 @@
         <v/>
       </c>
       <c r="H240" s="35" t="e">
-        <f>$F240/$G240</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I240" t="e">
@@ -32061,7 +32130,7 @@
         <v/>
       </c>
       <c r="H241" s="35" t="e">
-        <f>$F241/$G241</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I241" t="e">
@@ -32080,7 +32149,7 @@
         <v/>
       </c>
       <c r="H242" s="35" t="e">
-        <f>$F242/$G242</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I242" t="e">
@@ -32099,7 +32168,7 @@
         <v/>
       </c>
       <c r="H243" s="35" t="e">
-        <f>$F243/$G243</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I243" t="e">
@@ -32118,7 +32187,7 @@
         <v/>
       </c>
       <c r="H244" s="35" t="e">
-        <f>$F244/$G244</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I244" t="e">
@@ -32137,7 +32206,7 @@
         <v/>
       </c>
       <c r="H245" s="35" t="e">
-        <f>$F245/$G245</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I245" t="e">
@@ -32156,7 +32225,7 @@
         <v/>
       </c>
       <c r="H246" s="35" t="e">
-        <f>$F246/$G246</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I246" t="e">
@@ -32175,7 +32244,7 @@
         <v/>
       </c>
       <c r="H247" s="35" t="e">
-        <f>$F247/$G247</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I247" t="e">
@@ -32194,7 +32263,7 @@
         <v/>
       </c>
       <c r="H248" s="35" t="e">
-        <f>$F248/$G248</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I248" t="e">
@@ -32213,7 +32282,7 @@
         <v/>
       </c>
       <c r="H249" s="35" t="e">
-        <f>$F249/$G249</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I249" t="e">
@@ -32232,7 +32301,7 @@
         <v/>
       </c>
       <c r="H250" s="35" t="e">
-        <f>$F250/$G250</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I250" t="e">
@@ -32251,7 +32320,7 @@
         <v/>
       </c>
       <c r="H251" s="35" t="e">
-        <f>$F251/$G251</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I251" t="e">
@@ -32270,7 +32339,7 @@
         <v/>
       </c>
       <c r="H252" s="35" t="e">
-        <f>$F252/$G252</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I252" t="e">
@@ -32289,7 +32358,7 @@
         <v/>
       </c>
       <c r="H253" s="35" t="e">
-        <f>$F253/$G253</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I253" t="e">
@@ -32308,7 +32377,7 @@
         <v/>
       </c>
       <c r="H254" s="35" t="e">
-        <f>$F254/$G254</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I254" t="e">
@@ -32327,7 +32396,7 @@
         <v/>
       </c>
       <c r="H255" s="35" t="e">
-        <f>$F255/$G255</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I255" t="e">
@@ -32346,7 +32415,7 @@
         <v/>
       </c>
       <c r="H256" s="35" t="e">
-        <f>$F256/$G256</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I256" t="e">
@@ -32365,7 +32434,7 @@
         <v/>
       </c>
       <c r="H257" s="35" t="e">
-        <f>$F257/$G257</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I257" t="e">
@@ -32384,7 +32453,7 @@
         <v/>
       </c>
       <c r="H258" s="35" t="e">
-        <f>$F258/$G258</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I258" t="e">
@@ -32403,7 +32472,7 @@
         <v/>
       </c>
       <c r="H259" s="35" t="e">
-        <f>$F259/$G259</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I259" t="e">
@@ -32422,7 +32491,7 @@
         <v/>
       </c>
       <c r="H260" s="35" t="e">
-        <f>$F260/$G260</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I260" t="e">
@@ -32441,7 +32510,7 @@
         <v/>
       </c>
       <c r="H261" s="35" t="e">
-        <f>$F261/$G261</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I261" t="e">
@@ -32460,7 +32529,7 @@
         <v/>
       </c>
       <c r="H262" s="35" t="e">
-        <f>$F262/$G262</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I262" t="e">
@@ -32479,7 +32548,7 @@
         <v/>
       </c>
       <c r="H263" s="35" t="e">
-        <f>$F263/$G263</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I263" t="e">
@@ -32498,7 +32567,7 @@
         <v/>
       </c>
       <c r="H264" s="35" t="e">
-        <f>$F264/$G264</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I264" t="e">
@@ -32517,7 +32586,7 @@
         <v/>
       </c>
       <c r="H265" s="35" t="e">
-        <f>$F265/$G265</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I265" t="e">
@@ -32536,7 +32605,7 @@
         <v/>
       </c>
       <c r="H266" s="35" t="e">
-        <f>$F266/$G266</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I266" t="e">
@@ -32555,7 +32624,7 @@
         <v/>
       </c>
       <c r="H267" s="35" t="e">
-        <f>$F267/$G267</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I267" t="e">
@@ -32574,7 +32643,7 @@
         <v/>
       </c>
       <c r="H268" s="35" t="e">
-        <f>$F268/$G268</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I268" t="e">
@@ -32593,7 +32662,7 @@
         <v/>
       </c>
       <c r="H269" s="35" t="e">
-        <f>$F269/$G269</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I269" t="e">
@@ -32612,7 +32681,7 @@
         <v/>
       </c>
       <c r="H270" s="35" t="e">
-        <f>$F270/$G270</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I270" t="e">
@@ -32631,7 +32700,7 @@
         <v/>
       </c>
       <c r="H271" s="35" t="e">
-        <f>$F271/$G271</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I271" t="e">
@@ -32650,7 +32719,7 @@
         <v/>
       </c>
       <c r="H272" s="35" t="e">
-        <f>$F272/$G272</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I272" t="e">
@@ -32669,7 +32738,7 @@
         <v/>
       </c>
       <c r="H273" s="35" t="e">
-        <f>$F273/$G273</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I273" t="e">
@@ -32688,7 +32757,7 @@
         <v/>
       </c>
       <c r="H274" s="35" t="e">
-        <f>$F274/$G274</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I274" t="e">
@@ -32707,7 +32776,7 @@
         <v/>
       </c>
       <c r="H275" s="35" t="e">
-        <f>$F275/$G275</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I275" t="e">
@@ -32726,7 +32795,7 @@
         <v/>
       </c>
       <c r="H276" s="35" t="e">
-        <f>$F276/$G276</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I276" t="e">
@@ -32745,7 +32814,7 @@
         <v/>
       </c>
       <c r="H277" s="35" t="e">
-        <f>$F277/$G277</f>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I277" t="e">
@@ -32764,7 +32833,7 @@
         <v/>
       </c>
       <c r="H278" s="35" t="e">
-        <f>$F278/$G278</f>
+        <f t="shared" ref="H278:H341" si="6">$F278/$G278</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I278" t="e">
@@ -32783,7 +32852,7 @@
         <v/>
       </c>
       <c r="H279" s="35" t="e">
-        <f>$F279/$G279</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I279" t="e">
@@ -32802,7 +32871,7 @@
         <v/>
       </c>
       <c r="H280" s="35" t="e">
-        <f>$F280/$G280</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I280" t="e">
@@ -32821,7 +32890,7 @@
         <v/>
       </c>
       <c r="H281" s="35" t="e">
-        <f>$F281/$G281</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I281" t="e">
@@ -32840,7 +32909,7 @@
         <v/>
       </c>
       <c r="H282" s="35" t="e">
-        <f>$F282/$G282</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I282" t="e">
@@ -32859,7 +32928,7 @@
         <v/>
       </c>
       <c r="H283" s="35" t="e">
-        <f>$F283/$G283</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I283" t="e">
@@ -32878,7 +32947,7 @@
         <v/>
       </c>
       <c r="H284" s="35" t="e">
-        <f>$F284/$G284</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I284" t="e">
@@ -32897,7 +32966,7 @@
         <v/>
       </c>
       <c r="H285" s="35" t="e">
-        <f>$F285/$G285</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I285" t="e">
@@ -32916,7 +32985,7 @@
         <v/>
       </c>
       <c r="H286" s="35" t="e">
-        <f>$F286/$G286</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I286" t="e">
@@ -32935,7 +33004,7 @@
         <v/>
       </c>
       <c r="H287" s="35" t="e">
-        <f>$F287/$G287</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I287" t="e">
@@ -32954,7 +33023,7 @@
         <v/>
       </c>
       <c r="H288" s="35" t="e">
-        <f>$F288/$G288</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I288" t="e">
@@ -32973,7 +33042,7 @@
         <v/>
       </c>
       <c r="H289" s="35" t="e">
-        <f>$F289/$G289</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I289" t="e">
@@ -32992,7 +33061,7 @@
         <v/>
       </c>
       <c r="H290" s="35" t="e">
-        <f>$F290/$G290</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I290" t="e">
@@ -33011,7 +33080,7 @@
         <v/>
       </c>
       <c r="H291" s="35" t="e">
-        <f>$F291/$G291</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I291" t="e">
@@ -33030,7 +33099,7 @@
         <v/>
       </c>
       <c r="H292" s="35" t="e">
-        <f>$F292/$G292</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I292" t="e">
@@ -33049,7 +33118,7 @@
         <v/>
       </c>
       <c r="H293" s="35" t="e">
-        <f>$F293/$G293</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I293" t="e">
@@ -33068,7 +33137,7 @@
         <v/>
       </c>
       <c r="H294" s="35" t="e">
-        <f>$F294/$G294</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I294" t="e">
@@ -33087,7 +33156,7 @@
         <v/>
       </c>
       <c r="H295" s="35" t="e">
-        <f>$F295/$G295</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I295" t="e">
@@ -33106,7 +33175,7 @@
         <v/>
       </c>
       <c r="H296" s="35" t="e">
-        <f>$F296/$G296</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I296" t="e">
@@ -33125,7 +33194,7 @@
         <v/>
       </c>
       <c r="H297" s="35" t="e">
-        <f>$F297/$G297</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I297" t="e">
@@ -33144,7 +33213,7 @@
         <v/>
       </c>
       <c r="H298" s="35" t="e">
-        <f>$F298/$G298</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I298" t="e">
@@ -33163,7 +33232,7 @@
         <v/>
       </c>
       <c r="H299" s="35" t="e">
-        <f>$F299/$G299</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I299" t="e">
@@ -33182,7 +33251,7 @@
         <v/>
       </c>
       <c r="H300" s="35" t="e">
-        <f>$F300/$G300</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I300" t="e">
@@ -33201,7 +33270,7 @@
         <v/>
       </c>
       <c r="H301" s="35" t="e">
-        <f>$F301/$G301</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I301" t="e">
@@ -33220,7 +33289,7 @@
         <v/>
       </c>
       <c r="H302" s="35" t="e">
-        <f>$F302/$G302</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I302" t="e">
@@ -33239,7 +33308,7 @@
         <v/>
       </c>
       <c r="H303" s="35" t="e">
-        <f>$F303/$G303</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I303" t="e">
@@ -33258,7 +33327,7 @@
         <v/>
       </c>
       <c r="H304" s="35" t="e">
-        <f>$F304/$G304</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I304" t="e">
@@ -33277,7 +33346,7 @@
         <v/>
       </c>
       <c r="H305" s="35" t="e">
-        <f>$F305/$G305</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I305" t="e">
@@ -33296,7 +33365,7 @@
         <v/>
       </c>
       <c r="H306" s="35" t="e">
-        <f>$F306/$G306</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I306" t="e">
@@ -33315,7 +33384,7 @@
         <v/>
       </c>
       <c r="H307" s="35" t="e">
-        <f>$F307/$G307</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I307" t="e">
@@ -33334,7 +33403,7 @@
         <v/>
       </c>
       <c r="H308" s="35" t="e">
-        <f>$F308/$G308</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I308" t="e">
@@ -33353,7 +33422,7 @@
         <v/>
       </c>
       <c r="H309" s="35" t="e">
-        <f>$F309/$G309</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I309" t="e">
@@ -33372,7 +33441,7 @@
         <v/>
       </c>
       <c r="H310" s="35" t="e">
-        <f>$F310/$G310</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I310" t="e">
@@ -33391,7 +33460,7 @@
         <v/>
       </c>
       <c r="H311" s="35" t="e">
-        <f>$F311/$G311</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I311" t="e">
@@ -33410,7 +33479,7 @@
         <v/>
       </c>
       <c r="H312" s="35" t="e">
-        <f>$F312/$G312</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I312" t="e">
@@ -33429,7 +33498,7 @@
         <v/>
       </c>
       <c r="H313" s="35" t="e">
-        <f>$F313/$G313</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I313" t="e">
@@ -33448,7 +33517,7 @@
         <v/>
       </c>
       <c r="H314" s="35" t="e">
-        <f>$F314/$G314</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I314" t="e">
@@ -33467,7 +33536,7 @@
         <v/>
       </c>
       <c r="H315" s="35" t="e">
-        <f>$F315/$G315</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I315" t="e">
@@ -33486,7 +33555,7 @@
         <v/>
       </c>
       <c r="H316" s="35" t="e">
-        <f>$F316/$G316</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I316" t="e">
@@ -33505,7 +33574,7 @@
         <v/>
       </c>
       <c r="H317" s="35" t="e">
-        <f>$F317/$G317</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I317" t="e">
@@ -33524,7 +33593,7 @@
         <v/>
       </c>
       <c r="H318" s="35" t="e">
-        <f>$F318/$G318</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I318" t="e">
@@ -33543,7 +33612,7 @@
         <v/>
       </c>
       <c r="H319" s="35" t="e">
-        <f>$F319/$G319</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I319" t="e">
@@ -33562,7 +33631,7 @@
         <v/>
       </c>
       <c r="H320" s="35" t="e">
-        <f>$F320/$G320</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I320" t="e">
@@ -33581,7 +33650,7 @@
         <v/>
       </c>
       <c r="H321" s="35" t="e">
-        <f>$F321/$G321</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I321" t="e">
@@ -33600,7 +33669,7 @@
         <v/>
       </c>
       <c r="H322" s="35" t="e">
-        <f>$F322/$G322</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I322" t="e">
@@ -33619,7 +33688,7 @@
         <v/>
       </c>
       <c r="H323" s="35" t="e">
-        <f>$F323/$G323</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I323" t="e">
@@ -33638,7 +33707,7 @@
         <v/>
       </c>
       <c r="H324" s="35" t="e">
-        <f>$F324/$G324</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I324" t="e">
@@ -33657,7 +33726,7 @@
         <v/>
       </c>
       <c r="H325" s="35" t="e">
-        <f>$F325/$G325</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I325" t="e">
@@ -33676,7 +33745,7 @@
         <v/>
       </c>
       <c r="H326" s="35" t="e">
-        <f>$F326/$G326</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I326" t="e">
@@ -33695,7 +33764,7 @@
         <v/>
       </c>
       <c r="H327" s="35" t="e">
-        <f>$F327/$G327</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I327" t="e">
@@ -33714,7 +33783,7 @@
         <v/>
       </c>
       <c r="H328" s="35" t="e">
-        <f>$F328/$G328</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I328" t="e">
@@ -33733,7 +33802,7 @@
         <v/>
       </c>
       <c r="H329" s="35" t="e">
-        <f>$F329/$G329</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I329" t="e">
@@ -33752,7 +33821,7 @@
         <v/>
       </c>
       <c r="H330" s="35" t="e">
-        <f>$F330/$G330</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I330" t="e">
@@ -33771,7 +33840,7 @@
         <v/>
       </c>
       <c r="H331" s="35" t="e">
-        <f>$F331/$G331</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I331" t="e">
@@ -33790,7 +33859,7 @@
         <v/>
       </c>
       <c r="H332" s="35" t="e">
-        <f>$F332/$G332</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I332" t="e">
@@ -33809,7 +33878,7 @@
         <v/>
       </c>
       <c r="H333" s="35" t="e">
-        <f>$F333/$G333</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I333" t="e">
@@ -33828,7 +33897,7 @@
         <v/>
       </c>
       <c r="H334" s="35" t="e">
-        <f>$F334/$G334</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I334" t="e">
@@ -33847,7 +33916,7 @@
         <v/>
       </c>
       <c r="H335" s="35" t="e">
-        <f>$F335/$G335</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I335" t="e">
@@ -33866,7 +33935,7 @@
         <v/>
       </c>
       <c r="H336" s="35" t="e">
-        <f>$F336/$G336</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I336" t="e">
@@ -33885,7 +33954,7 @@
         <v/>
       </c>
       <c r="H337" s="35" t="e">
-        <f>$F337/$G337</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I337" t="e">
@@ -33904,7 +33973,7 @@
         <v/>
       </c>
       <c r="H338" s="35" t="e">
-        <f>$F338/$G338</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I338" t="e">
@@ -33923,7 +33992,7 @@
         <v/>
       </c>
       <c r="H339" s="35" t="e">
-        <f>$F339/$G339</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I339" t="e">
@@ -33942,7 +34011,7 @@
         <v/>
       </c>
       <c r="H340" s="35" t="e">
-        <f>$F340/$G340</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I340" t="e">
@@ -33961,7 +34030,7 @@
         <v/>
       </c>
       <c r="H341" s="35" t="e">
-        <f>$F341/$G341</f>
+        <f t="shared" si="6"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I341" t="e">
@@ -33980,7 +34049,7 @@
         <v/>
       </c>
       <c r="H342" s="35" t="e">
-        <f>$F342/$G342</f>
+        <f t="shared" ref="H342:H405" si="7">$F342/$G342</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I342" t="e">
@@ -33999,7 +34068,7 @@
         <v/>
       </c>
       <c r="H343" s="35" t="e">
-        <f>$F343/$G343</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I343" t="e">
@@ -34018,7 +34087,7 @@
         <v/>
       </c>
       <c r="H344" s="35" t="e">
-        <f>$F344/$G344</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I344" t="e">
@@ -34037,7 +34106,7 @@
         <v/>
       </c>
       <c r="H345" s="35" t="e">
-        <f>$F345/$G345</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I345" t="e">
@@ -34056,7 +34125,7 @@
         <v/>
       </c>
       <c r="H346" s="35" t="e">
-        <f>$F346/$G346</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I346" t="e">
@@ -34075,7 +34144,7 @@
         <v/>
       </c>
       <c r="H347" s="35" t="e">
-        <f>$F347/$G347</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I347" t="e">
@@ -34094,7 +34163,7 @@
         <v/>
       </c>
       <c r="H348" s="35" t="e">
-        <f>$F348/$G348</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I348" t="e">
@@ -34113,7 +34182,7 @@
         <v/>
       </c>
       <c r="H349" s="35" t="e">
-        <f>$F349/$G349</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I349" t="e">
@@ -34132,7 +34201,7 @@
         <v/>
       </c>
       <c r="H350" s="35" t="e">
-        <f>$F350/$G350</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I350" t="e">
@@ -34151,7 +34220,7 @@
         <v/>
       </c>
       <c r="H351" s="35" t="e">
-        <f>$F351/$G351</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I351" t="e">
@@ -34170,7 +34239,7 @@
         <v/>
       </c>
       <c r="H352" s="35" t="e">
-        <f>$F352/$G352</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I352" t="e">
@@ -34189,7 +34258,7 @@
         <v/>
       </c>
       <c r="H353" s="35" t="e">
-        <f>$F353/$G353</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I353" t="e">
@@ -34208,7 +34277,7 @@
         <v/>
       </c>
       <c r="H354" s="35" t="e">
-        <f>$F354/$G354</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I354" t="e">
@@ -34227,7 +34296,7 @@
         <v/>
       </c>
       <c r="H355" s="35" t="e">
-        <f>$F355/$G355</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I355" t="e">
@@ -34246,7 +34315,7 @@
         <v/>
       </c>
       <c r="H356" s="35" t="e">
-        <f>$F356/$G356</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I356" t="e">
@@ -34265,7 +34334,7 @@
         <v/>
       </c>
       <c r="H357" s="35" t="e">
-        <f>$F357/$G357</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I357" t="e">
@@ -34284,7 +34353,7 @@
         <v/>
       </c>
       <c r="H358" s="35" t="e">
-        <f>$F358/$G358</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I358" t="e">
@@ -34303,7 +34372,7 @@
         <v/>
       </c>
       <c r="H359" s="35" t="e">
-        <f>$F359/$G359</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I359" t="e">
@@ -34322,7 +34391,7 @@
         <v/>
       </c>
       <c r="H360" s="35" t="e">
-        <f>$F360/$G360</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I360" t="e">
@@ -34341,7 +34410,7 @@
         <v/>
       </c>
       <c r="H361" s="35" t="e">
-        <f>$F361/$G361</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I361" t="e">
@@ -34360,7 +34429,7 @@
         <v/>
       </c>
       <c r="H362" s="35" t="e">
-        <f>$F362/$G362</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I362" t="e">
@@ -34379,7 +34448,7 @@
         <v/>
       </c>
       <c r="H363" s="35" t="e">
-        <f>$F363/$G363</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I363" t="e">
@@ -34398,7 +34467,7 @@
         <v/>
       </c>
       <c r="H364" s="35" t="e">
-        <f>$F364/$G364</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I364" t="e">
@@ -34417,7 +34486,7 @@
         <v/>
       </c>
       <c r="H365" s="35" t="e">
-        <f>$F365/$G365</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I365" t="e">
@@ -34436,7 +34505,7 @@
         <v/>
       </c>
       <c r="H366" s="35" t="e">
-        <f>$F366/$G366</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I366" t="e">
@@ -34455,7 +34524,7 @@
         <v/>
       </c>
       <c r="H367" s="35" t="e">
-        <f>$F367/$G367</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I367" t="e">
@@ -34474,7 +34543,7 @@
         <v/>
       </c>
       <c r="H368" s="35" t="e">
-        <f>$F368/$G368</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I368" t="e">
@@ -34493,7 +34562,7 @@
         <v/>
       </c>
       <c r="H369" s="35" t="e">
-        <f>$F369/$G369</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I369" t="e">
@@ -34512,7 +34581,7 @@
         <v/>
       </c>
       <c r="H370" s="35" t="e">
-        <f>$F370/$G370</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I370" t="e">
@@ -34531,7 +34600,7 @@
         <v/>
       </c>
       <c r="H371" s="35" t="e">
-        <f>$F371/$G371</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I371" t="e">
@@ -34550,7 +34619,7 @@
         <v/>
       </c>
       <c r="H372" s="35" t="e">
-        <f>$F372/$G372</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I372" t="e">
@@ -34569,7 +34638,7 @@
         <v/>
       </c>
       <c r="H373" s="35" t="e">
-        <f>$F373/$G373</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I373" t="e">
@@ -34588,7 +34657,7 @@
         <v/>
       </c>
       <c r="H374" s="35" t="e">
-        <f>$F374/$G374</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I374" t="e">
@@ -34607,7 +34676,7 @@
         <v/>
       </c>
       <c r="H375" s="35" t="e">
-        <f>$F375/$G375</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I375" t="e">
@@ -34626,7 +34695,7 @@
         <v/>
       </c>
       <c r="H376" s="35" t="e">
-        <f>$F376/$G376</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I376" t="e">
@@ -34645,7 +34714,7 @@
         <v/>
       </c>
       <c r="H377" s="35" t="e">
-        <f>$F377/$G377</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I377" t="e">
@@ -34664,7 +34733,7 @@
         <v/>
       </c>
       <c r="H378" s="35" t="e">
-        <f>$F378/$G378</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I378" t="e">
@@ -34683,7 +34752,7 @@
         <v/>
       </c>
       <c r="H379" s="35" t="e">
-        <f>$F379/$G379</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I379" t="e">
@@ -34702,7 +34771,7 @@
         <v/>
       </c>
       <c r="H380" s="35" t="e">
-        <f>$F380/$G380</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I380" t="e">
@@ -34721,7 +34790,7 @@
         <v/>
       </c>
       <c r="H381" s="35" t="e">
-        <f>$F381/$G381</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I381" t="e">
@@ -34740,7 +34809,7 @@
         <v/>
       </c>
       <c r="H382" s="35" t="e">
-        <f>$F382/$G382</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I382" t="e">
@@ -34759,7 +34828,7 @@
         <v/>
       </c>
       <c r="H383" s="35" t="e">
-        <f>$F383/$G383</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I383" t="e">
@@ -34778,7 +34847,7 @@
         <v/>
       </c>
       <c r="H384" s="35" t="e">
-        <f>$F384/$G384</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I384" t="e">
@@ -34797,7 +34866,7 @@
         <v/>
       </c>
       <c r="H385" s="35" t="e">
-        <f>$F385/$G385</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I385" t="e">
@@ -34816,7 +34885,7 @@
         <v/>
       </c>
       <c r="H386" s="35" t="e">
-        <f>$F386/$G386</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I386" t="e">
@@ -34835,7 +34904,7 @@
         <v/>
       </c>
       <c r="H387" s="35" t="e">
-        <f>$F387/$G387</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I387" t="e">
@@ -34854,7 +34923,7 @@
         <v/>
       </c>
       <c r="H388" s="35" t="e">
-        <f>$F388/$G388</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I388" t="e">
@@ -34873,7 +34942,7 @@
         <v/>
       </c>
       <c r="H389" s="35" t="e">
-        <f>$F389/$G389</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I389" t="e">
@@ -34892,7 +34961,7 @@
         <v/>
       </c>
       <c r="H390" s="35" t="e">
-        <f>$F390/$G390</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I390" t="e">
@@ -34911,7 +34980,7 @@
         <v/>
       </c>
       <c r="H391" s="35" t="e">
-        <f>$F391/$G391</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I391" t="e">
@@ -34930,7 +34999,7 @@
         <v/>
       </c>
       <c r="H392" s="35" t="e">
-        <f>$F392/$G392</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I392" t="e">
@@ -34949,7 +35018,7 @@
         <v/>
       </c>
       <c r="H393" s="35" t="e">
-        <f>$F393/$G393</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I393" t="e">
@@ -34968,7 +35037,7 @@
         <v/>
       </c>
       <c r="H394" s="35" t="e">
-        <f>$F394/$G394</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I394" t="e">
@@ -34987,7 +35056,7 @@
         <v/>
       </c>
       <c r="H395" s="35" t="e">
-        <f>$F395/$G395</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I395" t="e">
@@ -35006,7 +35075,7 @@
         <v/>
       </c>
       <c r="H396" s="35" t="e">
-        <f>$F396/$G396</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I396" t="e">
@@ -35025,7 +35094,7 @@
         <v/>
       </c>
       <c r="H397" s="35" t="e">
-        <f>$F397/$G397</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I397" t="e">
@@ -35044,7 +35113,7 @@
         <v/>
       </c>
       <c r="H398" s="35" t="e">
-        <f>$F398/$G398</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I398" t="e">
@@ -35063,7 +35132,7 @@
         <v/>
       </c>
       <c r="H399" s="35" t="e">
-        <f>$F399/$G399</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I399" t="e">
@@ -35082,7 +35151,7 @@
         <v/>
       </c>
       <c r="H400" s="35" t="e">
-        <f>$F400/$G400</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I400" t="e">
@@ -35101,7 +35170,7 @@
         <v/>
       </c>
       <c r="H401" s="35" t="e">
-        <f>$F401/$G401</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I401" t="e">
@@ -35120,7 +35189,7 @@
         <v/>
       </c>
       <c r="H402" s="35" t="e">
-        <f>$F402/$G402</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I402" t="e">
@@ -35139,7 +35208,7 @@
         <v/>
       </c>
       <c r="H403" s="35" t="e">
-        <f>$F403/$G403</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I403" t="e">
@@ -35158,7 +35227,7 @@
         <v/>
       </c>
       <c r="H404" s="35" t="e">
-        <f>$F404/$G404</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I404" t="e">
@@ -35177,7 +35246,7 @@
         <v/>
       </c>
       <c r="H405" s="35" t="e">
-        <f>$F405/$G405</f>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I405" t="e">
@@ -35196,7 +35265,7 @@
         <v/>
       </c>
       <c r="H406" s="35" t="e">
-        <f>$F406/$G406</f>
+        <f t="shared" ref="H406:H433" si="8">$F406/$G406</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I406" t="e">
@@ -35215,7 +35284,7 @@
         <v/>
       </c>
       <c r="H407" s="35" t="e">
-        <f>$F407/$G407</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I407" t="e">
@@ -35234,7 +35303,7 @@
         <v/>
       </c>
       <c r="H408" s="35" t="e">
-        <f>$F408/$G408</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I408" t="e">
@@ -35253,7 +35322,7 @@
         <v/>
       </c>
       <c r="H409" s="35" t="e">
-        <f>$F409/$G409</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I409" t="e">
@@ -35272,7 +35341,7 @@
         <v/>
       </c>
       <c r="H410" s="35" t="e">
-        <f>$F410/$G410</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I410" t="e">
@@ -35291,7 +35360,7 @@
         <v/>
       </c>
       <c r="H411" s="35" t="e">
-        <f>$F411/$G411</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I411" t="e">
@@ -35310,7 +35379,7 @@
         <v/>
       </c>
       <c r="H412" s="35" t="e">
-        <f>$F412/$G412</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I412" t="e">
@@ -35329,7 +35398,7 @@
         <v/>
       </c>
       <c r="H413" s="35" t="e">
-        <f>$F413/$G413</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I413" t="e">
@@ -35348,7 +35417,7 @@
         <v/>
       </c>
       <c r="H414" s="35" t="e">
-        <f>$F414/$G414</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I414" t="e">
@@ -35367,7 +35436,7 @@
         <v/>
       </c>
       <c r="H415" s="35" t="e">
-        <f>$F415/$G415</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I415" t="e">
@@ -35386,7 +35455,7 @@
         <v/>
       </c>
       <c r="H416" s="35" t="e">
-        <f>$F416/$G416</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I416" t="e">
@@ -35405,7 +35474,7 @@
         <v/>
       </c>
       <c r="H417" s="35" t="e">
-        <f>$F417/$G417</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I417" t="e">
@@ -35424,7 +35493,7 @@
         <v/>
       </c>
       <c r="H418" s="35" t="e">
-        <f>$F418/$G418</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I418" t="e">
@@ -35443,7 +35512,7 @@
         <v/>
       </c>
       <c r="H419" s="35" t="e">
-        <f>$F419/$G419</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I419" t="e">
@@ -35462,7 +35531,7 @@
         <v/>
       </c>
       <c r="H420" s="35" t="e">
-        <f>$F420/$G420</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I420" t="e">
@@ -35481,7 +35550,7 @@
         <v/>
       </c>
       <c r="H421" s="35" t="e">
-        <f>$F421/$G421</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I421" t="e">
@@ -35500,7 +35569,7 @@
         <v/>
       </c>
       <c r="H422" s="35" t="e">
-        <f>$F422/$G422</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I422" t="e">
@@ -35519,7 +35588,7 @@
         <v/>
       </c>
       <c r="H423" s="35" t="e">
-        <f>$F423/$G423</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I423" t="e">
@@ -35538,7 +35607,7 @@
         <v/>
       </c>
       <c r="H424" s="35" t="e">
-        <f>$F424/$G424</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I424" t="e">
@@ -35557,7 +35626,7 @@
         <v/>
       </c>
       <c r="H425" s="35" t="e">
-        <f>$F425/$G425</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I425" t="e">
@@ -35576,7 +35645,7 @@
         <v/>
       </c>
       <c r="H426" s="35" t="e">
-        <f>$F426/$G426</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I426" t="e">
@@ -35595,7 +35664,7 @@
         <v/>
       </c>
       <c r="H427" s="35" t="e">
-        <f>$F427/$G427</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I427" t="e">
@@ -35614,7 +35683,7 @@
         <v/>
       </c>
       <c r="H428" s="35" t="e">
-        <f>$F428/$G428</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I428" t="e">
@@ -35633,7 +35702,7 @@
         <v/>
       </c>
       <c r="H429" s="35" t="e">
-        <f>$F429/$G429</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I429" t="e">
@@ -35652,7 +35721,7 @@
         <v/>
       </c>
       <c r="H430" s="35" t="e">
-        <f>$F430/$G430</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I430" t="e">
@@ -35671,7 +35740,7 @@
         <v/>
       </c>
       <c r="H431" s="35" t="e">
-        <f>$F431/$G431</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I431" t="e">
@@ -35690,7 +35759,7 @@
         <v/>
       </c>
       <c r="H432" s="35" t="e">
-        <f>$F432/$G432</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I432" t="e">
@@ -35709,7 +35778,7 @@
         <v/>
       </c>
       <c r="H433" s="35" t="e">
-        <f>$F433/$G433</f>
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
       <c r="I433" t="e">
@@ -35957,6 +36026,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="97003019-d0ea-4b44-a32d-a1d0fc52ffd7" xsi:nil="true"/>
@@ -35965,15 +36043,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35996,6 +36065,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E919C03E-5A89-47CF-BA2C-50B5836FBD2A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F22229DF-FCAD-420A-8F03-88F31FF2AFD8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -36010,12 +36087,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E919C03E-5A89-47CF-BA2C-50B5836FBD2A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>